<commit_message>
Update data dictionary columns and include Student_ID details in cleaning log
</commit_message>
<xml_diff>
--- a/Data Dictionary.xlsx
+++ b/Data Dictionary.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,46 +27,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="001F4E78"/>
-      <sz val="14"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-        <bgColor rgb="001F4E78"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2F6F9"/>
-        <bgColor rgb="00F2F6F9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -78,41 +47,20 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="00D3D3D3"/>
-      </left>
-      <right style="thin">
-        <color rgb="00D3D3D3"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D3D3D3"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D3D3D3"/>
-      </bottom>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -478,18 +426,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="29" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Nama Kolom</t>
@@ -497,571 +437,751 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Tipe Data</t>
+          <t>Jenis Data</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Tipe Data Detail</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Rentang Nilai</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Kategori</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Definisi Bisnis</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Keterangan Kualitas Data</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Cara Penanganan Kualitas Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Student_ID</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Text / Numeric</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Numerik</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
           <t>100001 - 150000</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Identitas &amp; Profil Akademik</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>ID unik mahasiswa pengenal catatan data.</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Terdapat 2 records korup/terbungkus kutip ganda di raw data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Terdapat 2 baris korup/terbungkus kutip ganda di raw data.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Perbaikan parsing kutip ganda secara terprogram, kemudian dikonversi ke tipe data Int64.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Major_Category</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Text (Categorical)</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Kategorik</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
         <is>
           <t>STEM, Business, Humanities, Medical, Arts</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Identitas &amp; Profil Akademik</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Rumpun program studi yang diambil oleh mahasiswa.</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>Terdapat 2 missing values.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Terdapat 2 missing values sebelum perbaikan parsing.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Baris teratasi otomatis setelah perbaikan parsing kutip ganda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Year_of_Study</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Text (Categorical)</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Kategorik</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
         <is>
           <t>Freshman, Sophomore, Junior, Senior, Graduate</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Identitas &amp; Profil Akademik</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Tingkat/tahun akademik studi mahasiswa.</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Terdapat 1 record bernilai tidak valid '123' dan 2 missing values.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Terdapat 1 record bernilai tidak valid '123' dan 2 missing values sebelum parsing.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Hapus 1 baris bernilai '123' (Student_ID: 127687). Missing values teratasi setelah parsing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Pre_Semester_GPA</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Decimal (Numeric)</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Numerik</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Desimal</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
         <is>
           <t>1.00 - 4.00</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Identitas &amp; Profil Akademik</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Indeks Prestasi Kumulatif (IPK) sebelum semester berjalan dimulai.</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>Terdapat 1 outlier bernilai &gt; 4.00 (12.249) dan 2 missing values.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Terdapat 1 outlier bernilai &gt; 4.00 (12.249) dan 2 missing values sebelum parsing.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Hapus 1 baris pencilan &gt; 4.00 (Student_ID: 145219). Missing values teratasi setelah parsing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Weekly_GenAI_Hours</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Decimal (Numeric)</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Numerik</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Desimal</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
         <is>
           <t>0.00 - 40.00</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Perilaku Penggunaan AI</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Rata-rata waktu penggunaan AI Generatif per minggu (dalam jam).</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Terdapat 2 missing values.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Terdapat 2 missing values sebelum parsing.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Teratasi otomatis setelah perbaikan parsing kutip ganda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Primary_Use_Case</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Text (Categorical)</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Kategorik</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
         <is>
           <t>Copywriting/Drafting, Summarizing_Reading, Debugging/Troubleshooting, Ideation, Direct_Answer_Generation</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Perilaku Penggunaan AI</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Tujuan utama mahasiswa dalam memanfaatkan AI Generatif.</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>Terdapat 2 missing values.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Terdapat 2 missing values sebelum parsing, tersisa 1 baris kosong setelah parsing.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Imputasi nilai kosong dengan modus ('Debugging/Troubleshooting') pada Student_ID: 100465.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Prompt_Engineering_Skill</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Text (Categorical)</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Kategorik</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
         <is>
           <t>Beginner, Intermediate, Advanced</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Perilaku Penggunaan AI</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Tingkat kemahiran mahasiswa dalam merancang instruksi (prompt) untuk AI.</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>Terdapat 2 missing values.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Terdapat 2 missing values sebelum parsing.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Teratasi otomatis setelah perbaikan parsing kutip ganda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Tool_Diversity</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Integer (Numeric)</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Numerik</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
         <is>
           <t>1 - 5</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>Perilaku Penggunaan AI</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Jumlah variasi aplikasi/sistem AI Generatif berbeda yang digunakan.</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>Terdapat 1 outlier bernilai &gt; 5 (18.0) dan 2 missing values.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Terdapat 1 outlier bernilai &gt; 5 (18.0) dan 2 missing values sebelum parsing.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Hapus 1 baris pencilan &gt; 5 (Student_ID: 100297). Missing values teratasi setelah parsing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Paid_Subscription</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Boolean (True/False)</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Kategorik</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Boolean</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
         <is>
           <t>True, False</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Perilaku Penggunaan AI</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Status kepemilikan langganan AI berbayar (Premium/Plus).</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>Mengandung mixed data types (string/Boolean) dan 2 missing values.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Mengandung mixed data types (string/Boolean) dan 2 missing values sebelum parsing.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Normalisasi data string 'True'/'False' menjadi tipe Boolean asli. Missing values teratasi setelah parsing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Traditional_Study_Hours</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Decimal (Numeric)</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Numerik</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Desimal</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
         <is>
           <t>1.00 - 36.00</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>Perilaku Belajar</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>Jam belajar mandiri secara tradisional (non-AI) per minggu.</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>Terdapat 2 missing values.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Terdapat 2 missing values sebelum parsing.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Teratasi otomatis setelah perbaikan parsing kutip ganda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Perceived_AI_Dependency</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Integer (Numeric)</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Numerik</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
         <is>
           <t>1 - 10</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Perilaku Belajar</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Skor persepsi tingkat ketergantungan mahasiswa terhadap AI (1=Sangat Rendah, 10=Sangat Tinggi).</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>Terdapat 2 missing values.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Terdapat 2 missing values sebelum parsing.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Teratasi otomatis setelah perbaikan parsing kutip ganda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Institutional_Policy</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Text (Categorical)</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Kategorik</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
         <is>
           <t>Allowed_With_Citation, Strict_Ban, Actively_Encouraged</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>Kebijakan Institusi</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>Regulasi yang diterapkan oleh perguruan tinggi terkait penggunaan AI.</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>Terdapat 2 missing values.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Terdapat 2 missing values sebelum parsing.</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Teratasi otomatis setelah perbaikan parsing kutip ganda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Anxiety_Level_During_Exams</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Integer (Numeric)</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Numerik</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
         <is>
           <t>1 - 10</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>Kesehatan Mental &amp; Kesejahteraan</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>Tingkat kecemasan mahasiswa saat menghadapi ujian (1=Sangat Rendah, 10=Sangat Tinggi).</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>Terdapat 2 missing values.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Terdapat 2 missing values sebelum parsing.</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Teratasi otomatis setelah perbaikan parsing kutip ganda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Post_Semester_GPA</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Decimal (Numeric)</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Numerik</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Desimal</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
         <is>
           <t>1.00 - 4.00</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>Identitas &amp; Profil Akademik</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>Indeks Prestasi Kumulatif (IPK) di akhir semester berjalan (variabel output utama).</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>Terdapat 1 outlier bernilai &gt; 4.00 (10.389) dan 2 missing values.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Terdapat 1 outlier bernilai &gt; 4.00 (10.389), 2 missing values sebelum parsing, tersisa 1 baris kosong setelah parsing.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Hapus 1 baris kosong target (Student_ID: 145825) dan hapus 1 baris pencilan &gt; 4.00 (Student_ID: 100089).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Skill_Retention_Score</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Decimal (Numeric)</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Numerik</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Desimal</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
         <is>
           <t>0.00 - 100.00</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>Kesehatan Mental &amp; Kesejahteraan</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>Skor retensi pemahaman materi kuliah pasca-semester berakhir.</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>Terdapat 2 missing values.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Terdapat 2 missing values sebelum parsing.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Teratasi otomatis setelah perbaikan parsing kutip ganda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Burnout_Risk_Level</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Text (Categorical)</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Kategorik</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
         <is>
           <t>Low, Medium, High</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>Kesehatan Mental &amp; Kesejahteraan</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>Klasifikasi tingkat risiko kelelahan fisik dan mental (burnout) mahasiswa.</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>Terdapat 2 missing values.</t>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Terdapat 2 missing values sebelum parsing.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Teratasi otomatis setelah perbaikan parsing kutip ganda.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>AI_Usage_Segment</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Text (Categorical)</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Kategorik</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
         <is>
           <t>Light User, Moderate User, Heavy User</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>Perilaku Penggunaan AI</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>Segmentasi intensitas penggunaan AI per minggu hasil rekayasa fitur dari Weekly_GenAI_Hours. Light: &lt;10 jam, Moderate: 10-20 jam, Heavy: &gt;20 jam.</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>Kolom baru hasil feature engineering (tidak ada di raw dataset). Tidak memiliki missing values.</t>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Kolom baru hasil feature engineering (tidak ada di raw dataset).</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Dihasilkan dari pengelompokan logis nilai Weekly_GenAI_Hours. Tidak memiliki missing values.</t>
         </is>
       </c>
     </row>
@@ -1078,185 +1198,194 @@
   </sheetPr>
   <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1">
-      <c r="A1" s="6" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Ringkasan Profiling Awal Dataset</t>
         </is>
       </c>
-    </row>
-    <row r="2"/>
-    <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 1</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Metrik Kualitas / Profiling</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Nilai / Status</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Keterangan Bisnis &amp; Rencana Tindak Lanjut</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Ukuran Baris (Records)</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>50.000</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Total responden mahasiswa dalam satu semester.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Ukuran Kolom (Variabel)</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>17</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Variabel profil akademik, penggunaan AI, belajar, kebijakan, dan mental.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Jumlah Duplikat</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Tidak terdeteksi baris data duplikat.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Jumlah Missing Values (Rata-rata per Kolom)</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Hampir seluruh kolom memiliki 2 missing values karena masalah parsing.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Jumlah Baris Korup / Cacat Parsing</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Student_ID 100465 dan 145825 terbungkus tanda kutip ganda sehingga terbaca 1 string.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Outlier Nilai IPK (GPA &gt; 4.00)</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Pre_Semester_GPA (12.249) dan Post_Semester_GPA (10.389) tidak logis.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Outlier Keragaman Alat (Tool_Diversity &gt; 5)</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Terdapat nilai 18 yang melebihi batas deskripsi instrumen (1-5).</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Nilai Invalid Tahun Studi (Year_of_Study)</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Terdapat nilai "123" pada salah satu responden.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Strategi Pembersihan Data</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Imputasi / Pembersihan Selektif</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Baris korup diperbaiki parsingnya, outlier di-drop atau diganti median/mean, missing values diimputasi.</t>
         </is>

</xml_diff>